<commit_message>
feat: dashboard concluído (4 páginas) e anonimização dos vendedores
</commit_message>
<xml_diff>
--- a/data/processed/positivacao/2020-01_positivacao_anonimizado.xlsx
+++ b/data/processed/positivacao/2020-01_positivacao_anonimizado.xlsx
@@ -551,7 +551,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Vendedor: 1 - ROBSON</t>
+          <t>Vendedor: 1 - VENDEDOR 01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -23775,7 +23775,7 @@
     <row r="902">
       <c r="A902" t="inlineStr">
         <is>
-          <t>Vendedor: 3 - FERNANDA</t>
+          <t>Vendedor: 3 - VENDEDOR 03</t>
         </is>
       </c>
       <c r="B902" t="inlineStr"/>
@@ -34971,7 +34971,7 @@
     <row r="1333">
       <c r="A1333" t="inlineStr">
         <is>
-          <t>Vendedor: 4 - DANIELA</t>
+          <t>Vendedor: 4 - VENDEDOR 04</t>
         </is>
       </c>
       <c r="B1333" t="inlineStr"/>
@@ -64019,7 +64019,7 @@
     <row r="2451">
       <c r="A2451" t="inlineStr">
         <is>
-          <t>Vendedor: 8 - RAFAEL</t>
+          <t>Vendedor: 8 - VENDEDOR 08</t>
         </is>
       </c>
       <c r="B2451" t="inlineStr"/>
@@ -65716,12 +65716,12 @@
       <c r="A2517" t="inlineStr"/>
       <c r="B2517" t="inlineStr">
         <is>
-          <t>Vendedor 1 - ROBSON: positivou 0 cliente(s), não positivou 93 cliente(s) - Total vendido: R$ 0,00
+          <t>Vendedor 1 - VENDEDOR 01: positivou 0 cliente(s), não positivou 93 cliente(s) - Total vendido: R$ 0,00
 Vendedor 18 - LOJA: positivou 1 cliente(s), não positivou 798 cliente(s) - Total vendido: R$ 3.000,00
-Vendedor 3 - FERNANDA: positivou 0 cliente(s), não positivou 430 cliente(s) - Total vendido: R$ 0,00
-Vendedor 4 - DANIELA: positivou 0 cliente(s), não positivou 661 cliente(s) - Total vendido: R$ 0,00
+Vendedor 3 - VENDEDOR 03: positivou 0 cliente(s), não positivou 430 cliente(s) - Total vendido: R$ 0,00
+Vendedor 4 - VENDEDOR 04: positivou 0 cliente(s), não positivou 661 cliente(s) - Total vendido: R$ 0,00
 Vendedor 5 - SITE: positivou 0 cliente(s), não positivou 455 cliente(s) - Total vendido: R$ 0,00
-Vendedor 8 - RAFAEL: positivou 0 cliente(s), não positivou 64 cliente(s) - Total vendido: R$ 0,00</t>
+Vendedor 8 - VENDEDOR 08: positivou 0 cliente(s), não positivou 64 cliente(s) - Total vendido: R$ 0,00</t>
         </is>
       </c>
       <c r="C2517" t="inlineStr"/>

</xml_diff>